<commit_message>
Spring 2026 updates v3
</commit_message>
<xml_diff>
--- a/src/data/current_data/bios_currentdata.xlsx
+++ b/src/data/current_data/bios_currentdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/riya/Desktop/dspuci-website-gatsby/dspuci-website-gatsby/src/data/current_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76C6E81-7CE6-9B47-81DB-55E7AED592FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5A860B-325D-7649-9734-770A9037B199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2740" yWindow="2920" windowWidth="24480" windowHeight="14540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1645,9 +1645,6 @@
     <t>Moraga, CA</t>
   </si>
   <si>
-    <t>Marketing Intern @ HawkRobo right</t>
-  </si>
-  <si>
     <t>Product Management, Project Management</t>
   </si>
   <si>
@@ -1655,6 +1652,9 @@
   </si>
   <si>
     <t>Product Association, Design @ UCI</t>
+  </si>
+  <si>
+    <t>Marketing Intern @ HawkRobo</t>
   </si>
 </sst>
 </file>
@@ -3133,13 +3133,13 @@
         <v>175</v>
       </c>
       <c r="J19" s="11" t="s">
+        <v>539</v>
+      </c>
+      <c r="K19" s="10" t="s">
         <v>540</v>
       </c>
-      <c r="K19" s="10" t="s">
+      <c r="L19" s="4" t="s">
         <v>541</v>
-      </c>
-      <c r="L19" s="4" t="s">
-        <v>542</v>
       </c>
       <c r="M19" s="4" t="s">
         <v>27</v>
@@ -4308,7 +4308,7 @@
         <v>366</v>
       </c>
       <c r="K41" s="11" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="L41" s="11" t="s">
         <v>74</v>

</xml_diff>